<commit_message>
adding augmentation strategy in dataset_config.py
</commit_message>
<xml_diff>
--- a/doc/stride_on_layers.xlsx
+++ b/doc/stride_on_layers.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t xml:space="preserve">Étape
 (Layer)</t>
@@ -38,13 +38,25 @@
     <t xml:space="preserve">Couverture d'1 seule cellule sur l'image d'origine (Receptive Field)</t>
   </si>
   <si>
+    <t xml:space="preserve">utilité</t>
+  </si>
+  <si>
     <t xml:space="preserve">Stage 0</t>
   </si>
   <si>
+    <t xml:space="preserve">L'étape 112x112 est le "décodeur bas niveau". Elle détecte les contours, les gradients, les lignes diagonales.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Stage 1</t>
   </si>
   <si>
+    <t xml:space="preserve">L'étape 56x56 assemble ces lignes pour comprendre des textures ou des formes simples (un bout de métal, un angle droit).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Stage 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'étape 28x28 assemble ces formes simples pour commencer à comprendre des concepts comme un bout d'aile ou une dérive.</t>
   </si>
   <si>
     <t xml:space="preserve">Stage 3 (feat_p3)</t>
@@ -60,7 +72,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -83,6 +95,11 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
@@ -136,7 +153,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -151,6 +168,18 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -336,10 +365,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultColWidth="15.859375" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="1" width="15.85"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="1" style="1" width="15.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="85.7"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="1" width="15.85"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -358,10 +389,13 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>224</v>
@@ -377,10 +411,13 @@
         <f aca="false">($B$2/D2)&amp;"x"&amp;($B$2/D2)</f>
         <v>2x2</v>
       </c>
+      <c r="F2" s="4" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B3" s="3" t="n">
         <f aca="false">D2</f>
@@ -397,10 +434,13 @@
         <f aca="false">($B$2/D3)&amp;"x"&amp;($B$2/D3)</f>
         <v>4x4</v>
       </c>
+      <c r="F3" s="5" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B4" s="3" t="n">
         <f aca="false">D3</f>
@@ -417,10 +457,13 @@
         <f aca="false">($B$2/D4)&amp;"x"&amp;($B$2/D4)</f>
         <v>8x8</v>
       </c>
+      <c r="F4" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B5" s="3" t="n">
         <f aca="false">D4</f>
@@ -437,10 +480,11 @@
         <f aca="false">($B$2/D5)&amp;"x"&amp;($B$2/D5)</f>
         <v>16x16</v>
       </c>
+      <c r="F5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B6" s="3" t="n">
         <f aca="false">D5</f>
@@ -457,6 +501,7 @@
         <f aca="false">($B$2/D6)&amp;"x"&amp;($B$2/D6)</f>
         <v>32x32</v>
       </c>
+      <c r="F6" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>